<commit_message>
Refactor data processing scripts to improve handling of exam columns and enhance photo data extraction
</commit_message>
<xml_diff>
--- a/app/data/RegentsCalendar.xlsx
+++ b/app/data/RegentsCalendar.xlsx
@@ -1,33 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/derekstampone/Library/Mobile Documents/com~apple~CloudDocs/Developer/data-specialist-flask/app/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A578EA1-53E3-6C4E-A067-E83ACCA3B152}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77BA4C98-77FF-A84C-9008-F7220D798498}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1700" yWindow="760" windowWidth="27880" windowHeight="18360" activeTab="2" xr2:uid="{98DCE2EE-096A-EF4C-9576-6BE138F05710}"/>
+    <workbookView xWindow="1800" yWindow="660" windowWidth="24620" windowHeight="18460" xr2:uid="{98DCE2EE-096A-EF4C-9576-6BE138F05710}"/>
   </bookViews>
   <sheets>
-    <sheet name="SectionProperties" sheetId="2" r:id="rId1"/>
-    <sheet name="SummerSectionProperties" sheetId="4" r:id="rId2"/>
-    <sheet name="2025-1" sheetId="6" r:id="rId3"/>
-    <sheet name="2024-7" sheetId="8" r:id="rId4"/>
-    <sheet name="2024-2" sheetId="7" r:id="rId5"/>
-    <sheet name="2024-1" sheetId="5" r:id="rId6"/>
-    <sheet name="2023-7" sheetId="3" r:id="rId7"/>
-    <sheet name="2023-2" sheetId="1" r:id="rId8"/>
+    <sheet name="2025-7" sheetId="9" r:id="rId1"/>
+    <sheet name="SectionProperties" sheetId="2" r:id="rId2"/>
+    <sheet name="SummerSectionProperties" sheetId="4" r:id="rId3"/>
+    <sheet name="2025-1" sheetId="6" r:id="rId4"/>
+    <sheet name="2024-7" sheetId="8" r:id="rId5"/>
+    <sheet name="2024-2" sheetId="7" r:id="rId6"/>
+    <sheet name="2024-1" sheetId="5" r:id="rId7"/>
+    <sheet name="2023-7" sheetId="3" r:id="rId8"/>
+    <sheet name="2023-2" sheetId="1" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'2023-2'!$A$1:$E$327</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'2023-7'!$A$1:$E$327</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'2024-2'!$A$1:$E$327</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'2024-7'!$A$1:$E$326</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">SummerSectionProperties!$A$1:$K$1004</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'2023-2'!$A$1:$E$327</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'2023-7'!$A$1:$E$327</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'2024-2'!$A$1:$E$327</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'2024-7'!$A$1:$E$326</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2025-7'!$A$1:$E$325</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">SummerSectionProperties!$A$1:$K$1004</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -50,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="195">
   <si>
     <t>Day</t>
   </si>
@@ -620,6 +622,21 @@
   </si>
   <si>
     <t>SJS43</t>
+  </si>
+  <si>
+    <t>EXRDG</t>
+  </si>
+  <si>
+    <t>MXRVG</t>
+  </si>
+  <si>
+    <t>SXR4G</t>
+  </si>
+  <si>
+    <t>Chem (new)</t>
+  </si>
+  <si>
+    <t>Chem (old)</t>
   </si>
 </sst>
 </file>
@@ -1059,6 +1076,258 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC2024DB-14EB-114C-B93B-2E1B671C0635}">
+  <dimension ref="A1:F263"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="13.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.5" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2" s="1">
+        <v>46252</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="8">
+        <v>1</v>
+      </c>
+      <c r="F2" s="12"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" s="1">
+        <v>46252</v>
+      </c>
+      <c r="B3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E3" s="8">
+        <v>2</v>
+      </c>
+      <c r="F3" s="12"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4" s="1">
+        <v>46252</v>
+      </c>
+      <c r="B4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E4" s="3">
+        <v>1</v>
+      </c>
+      <c r="F4" s="12"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" s="1">
+        <v>46252</v>
+      </c>
+      <c r="B5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6" s="1">
+        <v>46253</v>
+      </c>
+      <c r="B6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E6" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7" s="1">
+        <v>46253</v>
+      </c>
+      <c r="B7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="E7" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8" s="1">
+        <v>46253</v>
+      </c>
+      <c r="B8" t="s">
+        <v>2</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="E8" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9" s="1">
+        <v>46253</v>
+      </c>
+      <c r="B9" t="s">
+        <v>2</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="E9" s="3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10" s="1">
+        <v>46253</v>
+      </c>
+      <c r="B10" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E10" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A11" s="1">
+        <v>46253</v>
+      </c>
+      <c r="B11" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="E11" s="3">
+        <v>2</v>
+      </c>
+      <c r="F11" s="12"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A12" s="1"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+    </row>
+    <row r="216" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A216" s="2"/>
+      <c r="B216" s="2"/>
+    </row>
+    <row r="228" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A228" s="2"/>
+      <c r="B228" s="2"/>
+    </row>
+    <row r="229" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A229" s="2"/>
+      <c r="B229" s="2"/>
+    </row>
+    <row r="230" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A230" s="2"/>
+      <c r="B230" s="2"/>
+    </row>
+    <row r="231" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A231" s="2"/>
+      <c r="B231" s="2"/>
+    </row>
+    <row r="232" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A232" s="2"/>
+      <c r="B232" s="2"/>
+    </row>
+    <row r="235" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A235" s="2"/>
+      <c r="B235" s="2"/>
+    </row>
+    <row r="236" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A236" s="2"/>
+      <c r="B236" s="2"/>
+    </row>
+    <row r="263" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A263" s="2"/>
+      <c r="B263" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED29BD9C-93F7-3B47-BD2F-429330E86B98}">
   <dimension ref="A1:H1004"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -6277,7 +6546,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B6309B1-B2F2-C24D-9683-349831E0A64F}">
   <dimension ref="A1:V1004"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -14352,7 +14621,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DCA803E-0660-F641-BDDB-024EE43C3378}">
   <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -14612,7 +14881,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{517AF821-DE73-E44B-B05F-E5374FFCFDC2}">
   <dimension ref="A1:F264"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -14886,7 +15155,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52F52638-A0BD-4648-8682-FCD1751FE67B}">
   <dimension ref="A1:F265"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -15225,7 +15494,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF381A89-EC94-BD4E-AF94-947710DA3428}">
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -15426,7 +15695,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16B7BB07-9E9C-344A-8EF0-72CA0865EFBF}">
   <dimension ref="A1:E265"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -15636,7 +15905,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FB66886-AAD9-A442-BF69-AADD50D3EDBE}">
   <dimension ref="A1:E265"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>

</xml_diff>

<commit_message>
Refactor hub location logic and update registration processing; remove unused functions
</commit_message>
<xml_diff>
--- a/app/data/RegentsCalendar.xlsx
+++ b/app/data/RegentsCalendar.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/derekstampone/Library/Mobile Documents/com~apple~CloudDocs/Developer/data-specialist-flask/app/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/teacher/Developer/data-specialist-flask/app/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77BA4C98-77FF-A84C-9008-F7220D798498}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C000678E-5FF0-374D-B102-0567786B4DF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1800" yWindow="660" windowWidth="24620" windowHeight="18460" xr2:uid="{98DCE2EE-096A-EF4C-9576-6BE138F05710}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="34400" windowHeight="26380" xr2:uid="{98DCE2EE-096A-EF4C-9576-6BE138F05710}"/>
   </bookViews>
   <sheets>
     <sheet name="2025-7" sheetId="9" r:id="rId1"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="196">
   <si>
     <t>Day</t>
   </si>
@@ -637,6 +637,9 @@
   </si>
   <si>
     <t>Chem (old)</t>
+  </si>
+  <si>
+    <t>hub_location</t>
   </si>
 </sst>
 </file>
@@ -1104,6 +1107,9 @@
       <c r="E1" s="3" t="s">
         <v>173</v>
       </c>
+      <c r="F1" t="s">
+        <v>195</v>
+      </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
@@ -1121,7 +1127,9 @@
       <c r="E2" s="8">
         <v>1</v>
       </c>
-      <c r="F2" s="12"/>
+      <c r="F2" s="12">
+        <v>823</v>
+      </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
@@ -1139,7 +1147,9 @@
       <c r="E3" s="8">
         <v>2</v>
       </c>
-      <c r="F3" s="12"/>
+      <c r="F3" s="12">
+        <v>519</v>
+      </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
@@ -1157,7 +1167,9 @@
       <c r="E4" s="3">
         <v>1</v>
       </c>
-      <c r="F4" s="12"/>
+      <c r="F4" s="12">
+        <v>823</v>
+      </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
@@ -1175,6 +1187,9 @@
       <c r="E5" s="3">
         <v>2</v>
       </c>
+      <c r="F5" s="12">
+        <v>519</v>
+      </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
@@ -1192,6 +1207,9 @@
       <c r="E6" s="3">
         <v>1</v>
       </c>
+      <c r="F6" s="12">
+        <v>823</v>
+      </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
@@ -1209,6 +1227,9 @@
       <c r="E7" s="3">
         <v>2</v>
       </c>
+      <c r="F7" s="12">
+        <v>519</v>
+      </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
@@ -1226,6 +1247,9 @@
       <c r="E8" s="3">
         <v>2</v>
       </c>
+      <c r="F8" s="12">
+        <v>519</v>
+      </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
@@ -1243,6 +1267,9 @@
       <c r="E9" s="3">
         <v>3</v>
       </c>
+      <c r="F9" s="12">
+        <v>519</v>
+      </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
@@ -1260,6 +1287,9 @@
       <c r="E10" s="3">
         <v>1</v>
       </c>
+      <c r="F10" s="12">
+        <v>519</v>
+      </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
@@ -1277,7 +1307,9 @@
       <c r="E11" s="3">
         <v>2</v>
       </c>
-      <c r="F11" s="12"/>
+      <c r="F11" s="12">
+        <v>823</v>
+      </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="1"/>

</xml_diff>